<commit_message>
feat(calculators): finalise solution for calculating FA constant. Probably needs to be revisited
</commit_message>
<xml_diff>
--- a/packages/calculators/src/modules/test/5.2-organic-fertiliser.xlsx
+++ b/packages/calculators/src/modules/test/5.2-organic-fertiliser.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:20001_{67EA468A-9FC6-4247-B6BC-F4CABA8A56F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1720" yWindow="1780" windowWidth="46720" windowHeight="24460" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="5.2.1.1 (purchased_untraced)" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,6 @@
     <sheet name="5.2.1.1 (poultry)" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -38,7 +37,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -1432,7 +1431,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="168" formatCode="0.0000"/>
+    <numFmt numFmtId="164" formatCode="0.0000"/>
   </numFmts>
   <fonts count="6" x14ac:knownFonts="1">
     <font>
@@ -1507,21 +1506,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="168" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="168" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4875,7 +4873,7 @@
         <v>0.25</v>
       </c>
       <c r="W9">
-        <f t="shared" ref="W8:W17" si="17">IF(ISBLANK(K9),"", (R9*(1-S9-T9))-AB9)</f>
+        <f t="shared" ref="W9:W17" si="17">IF(ISBLANK(K9),"", (R9*(1-S9-T9))-AB9)</f>
         <v>3170.8421568000003</v>
       </c>
       <c r="X9">
@@ -11726,7 +11724,7 @@
         <v>0.2</v>
       </c>
       <c r="P43">
-        <f t="shared" ref="P43:P74" si="11">J43*O43</f>
+        <f t="shared" ref="P43:P70" si="11">J43*O43</f>
         <v>0.87688628970631199</v>
       </c>
       <c r="R43">
@@ -11754,7 +11752,7 @@
         <v>2.3454337149116478E-2</v>
       </c>
       <c r="X43">
-        <f t="shared" ref="X43:X74" si="17">(P43 / 6.25) - V43 - W43 - (1.1 * 10^-4 * POWER(E43,0.75) / 6.25)</f>
+        <f t="shared" ref="X43:X70" si="17">(P43 / 6.25) - V43 - W43 - (1.1 * 10^-4 * POWER(E43,0.75) / 6.25)</f>
         <v>0.10206990500776245</v>
       </c>
       <c r="Y43">
@@ -16050,7 +16048,7 @@
         <v>0.8</v>
       </c>
       <c r="J75">
-        <f t="shared" ref="J75:J106" si="18">(1.185 + 0.00454 * E75- 0.0000026 * E75^2 + 0.315 * I75)^2 * F75 + K75</f>
+        <f t="shared" ref="J75" si="18">(1.185 + 0.00454 * E75- 0.0000026 * E75^2 + 0.315 * I75)^2 * F75 + K75</f>
         <v>5.4143472656250013</v>
       </c>
       <c r="K75">
@@ -17812,7 +17810,7 @@
       <c r="Q10" s="1" t="s">
         <v>435</v>
       </c>
-      <c r="R10" s="8" t="s">
+      <c r="R10" t="s">
         <v>440</v>
       </c>
       <c r="U10" t="s">
@@ -17890,10 +17888,10 @@
       <c r="AU10" t="s">
         <v>3</v>
       </c>
-      <c r="AV10" s="9" t="s">
+      <c r="AV10" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="AW10" s="9" t="s">
+      <c r="AW10" s="7" t="s">
         <v>75</v>
       </c>
       <c r="BD10" s="4" t="s">
@@ -18778,7 +18776,7 @@
         <f>($AJ22*(1-$AK22-$AL22)-$AO22)*(1 -$B21)</f>
         <v>1.2820969691136002</v>
       </c>
-      <c r="AY22" s="6" t="s">
+      <c r="AY22" s="9" t="s">
         <v>404</v>
       </c>
       <c r="BA22" s="5"/>
@@ -18890,17 +18888,17 @@
         <f>($AJ23*(1-$AK23-$AL23)-$AO23)*(1 -$B21)</f>
         <v>80.224065750400001</v>
       </c>
-      <c r="AY23" s="6"/>
-      <c r="AZ23" s="7" t="s">
+      <c r="AY23" s="9"/>
+      <c r="AZ23" s="6" t="s">
         <v>405</v>
       </c>
-      <c r="BA23" s="7" t="s">
+      <c r="BA23" s="6" t="s">
         <v>415</v>
       </c>
-      <c r="BB23" s="7" t="s">
+      <c r="BB23" s="6" t="s">
         <v>416</v>
       </c>
-      <c r="BC23" s="7" t="s">
+      <c r="BC23" s="6" t="s">
         <v>406</v>
       </c>
     </row>
@@ -19072,16 +19070,16 @@
       <c r="AY26" s="5" t="s">
         <v>409</v>
       </c>
-      <c r="AZ26" s="11">
+      <c r="AZ26" s="8">
         <v>0.8</v>
       </c>
-      <c r="BA26" s="11">
+      <c r="BA26" s="8">
         <v>0.8</v>
       </c>
-      <c r="BB26" s="11">
+      <c r="BB26" s="8">
         <v>0.8</v>
       </c>
-      <c r="BC26" s="11">
+      <c r="BC26" s="8">
         <v>0.8</v>
       </c>
     </row>
@@ -19089,16 +19087,16 @@
       <c r="AY27" s="5" t="s">
         <v>410</v>
       </c>
-      <c r="AZ27" s="11">
+      <c r="AZ27" s="8">
         <v>0.19</v>
       </c>
-      <c r="BA27" s="11">
+      <c r="BA27" s="8">
         <v>0.23</v>
       </c>
-      <c r="BB27" s="11">
+      <c r="BB27" s="8">
         <v>0.19</v>
       </c>
-      <c r="BC27" s="11">
+      <c r="BC27" s="8">
         <v>0.23</v>
       </c>
     </row>
@@ -19106,16 +19104,16 @@
       <c r="AY28" s="5" t="s">
         <v>411</v>
       </c>
-      <c r="AZ28" s="11">
+      <c r="AZ28" s="8">
         <v>0.35</v>
       </c>
-      <c r="BA28" s="11">
+      <c r="BA28" s="8">
         <v>0.47</v>
       </c>
-      <c r="BB28" s="11">
+      <c r="BB28" s="8">
         <v>0.32</v>
       </c>
-      <c r="BC28" s="11">
+      <c r="BC28" s="8">
         <v>0.47</v>
       </c>
     </row>
@@ -19123,16 +19121,16 @@
       <c r="AY29" s="5" t="s">
         <v>412</v>
       </c>
-      <c r="AZ29" s="11">
+      <c r="AZ29" s="8">
         <v>0.18</v>
       </c>
-      <c r="BA29" s="11">
+      <c r="BA29" s="8">
         <v>0.15</v>
       </c>
-      <c r="BB29" s="11">
+      <c r="BB29" s="8">
         <v>0.18</v>
       </c>
-      <c r="BC29" s="11">
+      <c r="BC29" s="8">
         <v>0.15</v>
       </c>
     </row>

</xml_diff>

<commit_message>
4.1 beef pasture manure methane (#172)
* feat(calculators): first draft of beef pasture manure chapter 4.2, only partially done for now

* feat(calculators): first test case for beef pasture passing

* feat(calculators): method 2 for beef pasture manure passing test

* feat(calculators): finalise solution for calculating FA constant. Probably needs to be revisited
</commit_message>
<xml_diff>
--- a/packages/calculators/src/modules/test/5.2-organic-fertiliser.xlsx
+++ b/packages/calculators/src/modules/test/5.2-organic-fertiliser.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:20001_{67EA468A-9FC6-4247-B6BC-F4CABA8A56F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1720" yWindow="1780" windowWidth="46720" windowHeight="24460" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="5.2.1.1 (purchased_untraced)" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,6 @@
     <sheet name="5.2.1.1 (poultry)" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -38,7 +37,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -1432,7 +1431,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="168" formatCode="0.0000"/>
+    <numFmt numFmtId="164" formatCode="0.0000"/>
   </numFmts>
   <fonts count="6" x14ac:knownFonts="1">
     <font>
@@ -1507,21 +1506,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="168" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="168" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4875,7 +4873,7 @@
         <v>0.25</v>
       </c>
       <c r="W9">
-        <f t="shared" ref="W8:W17" si="17">IF(ISBLANK(K9),"", (R9*(1-S9-T9))-AB9)</f>
+        <f t="shared" ref="W9:W17" si="17">IF(ISBLANK(K9),"", (R9*(1-S9-T9))-AB9)</f>
         <v>3170.8421568000003</v>
       </c>
       <c r="X9">
@@ -11726,7 +11724,7 @@
         <v>0.2</v>
       </c>
       <c r="P43">
-        <f t="shared" ref="P43:P74" si="11">J43*O43</f>
+        <f t="shared" ref="P43:P70" si="11">J43*O43</f>
         <v>0.87688628970631199</v>
       </c>
       <c r="R43">
@@ -11754,7 +11752,7 @@
         <v>2.3454337149116478E-2</v>
       </c>
       <c r="X43">
-        <f t="shared" ref="X43:X74" si="17">(P43 / 6.25) - V43 - W43 - (1.1 * 10^-4 * POWER(E43,0.75) / 6.25)</f>
+        <f t="shared" ref="X43:X70" si="17">(P43 / 6.25) - V43 - W43 - (1.1 * 10^-4 * POWER(E43,0.75) / 6.25)</f>
         <v>0.10206990500776245</v>
       </c>
       <c r="Y43">
@@ -16050,7 +16048,7 @@
         <v>0.8</v>
       </c>
       <c r="J75">
-        <f t="shared" ref="J75:J106" si="18">(1.185 + 0.00454 * E75- 0.0000026 * E75^2 + 0.315 * I75)^2 * F75 + K75</f>
+        <f t="shared" ref="J75" si="18">(1.185 + 0.00454 * E75- 0.0000026 * E75^2 + 0.315 * I75)^2 * F75 + K75</f>
         <v>5.4143472656250013</v>
       </c>
       <c r="K75">
@@ -17812,7 +17810,7 @@
       <c r="Q10" s="1" t="s">
         <v>435</v>
       </c>
-      <c r="R10" s="8" t="s">
+      <c r="R10" t="s">
         <v>440</v>
       </c>
       <c r="U10" t="s">
@@ -17890,10 +17888,10 @@
       <c r="AU10" t="s">
         <v>3</v>
       </c>
-      <c r="AV10" s="9" t="s">
+      <c r="AV10" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="AW10" s="9" t="s">
+      <c r="AW10" s="7" t="s">
         <v>75</v>
       </c>
       <c r="BD10" s="4" t="s">
@@ -18778,7 +18776,7 @@
         <f>($AJ22*(1-$AK22-$AL22)-$AO22)*(1 -$B21)</f>
         <v>1.2820969691136002</v>
       </c>
-      <c r="AY22" s="6" t="s">
+      <c r="AY22" s="9" t="s">
         <v>404</v>
       </c>
       <c r="BA22" s="5"/>
@@ -18890,17 +18888,17 @@
         <f>($AJ23*(1-$AK23-$AL23)-$AO23)*(1 -$B21)</f>
         <v>80.224065750400001</v>
       </c>
-      <c r="AY23" s="6"/>
-      <c r="AZ23" s="7" t="s">
+      <c r="AY23" s="9"/>
+      <c r="AZ23" s="6" t="s">
         <v>405</v>
       </c>
-      <c r="BA23" s="7" t="s">
+      <c r="BA23" s="6" t="s">
         <v>415</v>
       </c>
-      <c r="BB23" s="7" t="s">
+      <c r="BB23" s="6" t="s">
         <v>416</v>
       </c>
-      <c r="BC23" s="7" t="s">
+      <c r="BC23" s="6" t="s">
         <v>406</v>
       </c>
     </row>
@@ -19072,16 +19070,16 @@
       <c r="AY26" s="5" t="s">
         <v>409</v>
       </c>
-      <c r="AZ26" s="11">
+      <c r="AZ26" s="8">
         <v>0.8</v>
       </c>
-      <c r="BA26" s="11">
+      <c r="BA26" s="8">
         <v>0.8</v>
       </c>
-      <c r="BB26" s="11">
+      <c r="BB26" s="8">
         <v>0.8</v>
       </c>
-      <c r="BC26" s="11">
+      <c r="BC26" s="8">
         <v>0.8</v>
       </c>
     </row>
@@ -19089,16 +19087,16 @@
       <c r="AY27" s="5" t="s">
         <v>410</v>
       </c>
-      <c r="AZ27" s="11">
+      <c r="AZ27" s="8">
         <v>0.19</v>
       </c>
-      <c r="BA27" s="11">
+      <c r="BA27" s="8">
         <v>0.23</v>
       </c>
-      <c r="BB27" s="11">
+      <c r="BB27" s="8">
         <v>0.19</v>
       </c>
-      <c r="BC27" s="11">
+      <c r="BC27" s="8">
         <v>0.23</v>
       </c>
     </row>
@@ -19106,16 +19104,16 @@
       <c r="AY28" s="5" t="s">
         <v>411</v>
       </c>
-      <c r="AZ28" s="11">
+      <c r="AZ28" s="8">
         <v>0.35</v>
       </c>
-      <c r="BA28" s="11">
+      <c r="BA28" s="8">
         <v>0.47</v>
       </c>
-      <c r="BB28" s="11">
+      <c r="BB28" s="8">
         <v>0.32</v>
       </c>
-      <c r="BC28" s="11">
+      <c r="BC28" s="8">
         <v>0.47</v>
       </c>
     </row>
@@ -19123,16 +19121,16 @@
       <c r="AY29" s="5" t="s">
         <v>412</v>
       </c>
-      <c r="AZ29" s="11">
+      <c r="AZ29" s="8">
         <v>0.18</v>
       </c>
-      <c r="BA29" s="11">
+      <c r="BA29" s="8">
         <v>0.15</v>
       </c>
-      <c r="BB29" s="11">
+      <c r="BB29" s="8">
         <v>0.18</v>
       </c>
-      <c r="BC29" s="11">
+      <c r="BC29" s="8">
         <v>0.15</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Revert "Merge branch 'feat/4.1-beef' into v4-15.2-purchased-feed"
This reverts commit 7a41ea696fb40f5992f7ab393558386b99275a1e, reversing
changes made to ef0a29006a1ffe12e6e772c45a376c46d1811d23.
</commit_message>
<xml_diff>
--- a/packages/calculators/src/modules/test/5.2-organic-fertiliser.xlsx
+++ b/packages/calculators/src/modules/test/5.2-organic-fertiliser.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:20001_{67EA468A-9FC6-4247-B6BC-F4CABA8A56F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1720" yWindow="1780" windowWidth="46720" windowHeight="24460" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="5.2.1.1 (purchased_untraced)" sheetId="1" r:id="rId1"/>
@@ -20,6 +20,7 @@
     <sheet name="5.2.1.1 (poultry)" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -1431,7 +1432,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="0.0000"/>
+    <numFmt numFmtId="168" formatCode="0.0000"/>
   </numFmts>
   <fonts count="6" x14ac:knownFonts="1">
     <font>
@@ -1506,20 +1507,21 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="168" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="168" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4873,7 +4875,7 @@
         <v>0.25</v>
       </c>
       <c r="W9">
-        <f t="shared" ref="W9:W17" si="17">IF(ISBLANK(K9),"", (R9*(1-S9-T9))-AB9)</f>
+        <f t="shared" ref="W8:W17" si="17">IF(ISBLANK(K9),"", (R9*(1-S9-T9))-AB9)</f>
         <v>3170.8421568000003</v>
       </c>
       <c r="X9">
@@ -11724,7 +11726,7 @@
         <v>0.2</v>
       </c>
       <c r="P43">
-        <f t="shared" ref="P43:P70" si="11">J43*O43</f>
+        <f t="shared" ref="P43:P74" si="11">J43*O43</f>
         <v>0.87688628970631199</v>
       </c>
       <c r="R43">
@@ -11752,7 +11754,7 @@
         <v>2.3454337149116478E-2</v>
       </c>
       <c r="X43">
-        <f t="shared" ref="X43:X70" si="17">(P43 / 6.25) - V43 - W43 - (1.1 * 10^-4 * POWER(E43,0.75) / 6.25)</f>
+        <f t="shared" ref="X43:X74" si="17">(P43 / 6.25) - V43 - W43 - (1.1 * 10^-4 * POWER(E43,0.75) / 6.25)</f>
         <v>0.10206990500776245</v>
       </c>
       <c r="Y43">
@@ -16048,7 +16050,7 @@
         <v>0.8</v>
       </c>
       <c r="J75">
-        <f t="shared" ref="J75" si="18">(1.185 + 0.00454 * E75- 0.0000026 * E75^2 + 0.315 * I75)^2 * F75 + K75</f>
+        <f t="shared" ref="J75:J106" si="18">(1.185 + 0.00454 * E75- 0.0000026 * E75^2 + 0.315 * I75)^2 * F75 + K75</f>
         <v>5.4143472656250013</v>
       </c>
       <c r="K75">
@@ -17810,7 +17812,7 @@
       <c r="Q10" s="1" t="s">
         <v>435</v>
       </c>
-      <c r="R10" t="s">
+      <c r="R10" s="8" t="s">
         <v>440</v>
       </c>
       <c r="U10" t="s">
@@ -17888,10 +17890,10 @@
       <c r="AU10" t="s">
         <v>3</v>
       </c>
-      <c r="AV10" s="7" t="s">
+      <c r="AV10" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="AW10" s="7" t="s">
+      <c r="AW10" s="9" t="s">
         <v>75</v>
       </c>
       <c r="BD10" s="4" t="s">
@@ -18776,7 +18778,7 @@
         <f>($AJ22*(1-$AK22-$AL22)-$AO22)*(1 -$B21)</f>
         <v>1.2820969691136002</v>
       </c>
-      <c r="AY22" s="9" t="s">
+      <c r="AY22" s="6" t="s">
         <v>404</v>
       </c>
       <c r="BA22" s="5"/>
@@ -18888,17 +18890,17 @@
         <f>($AJ23*(1-$AK23-$AL23)-$AO23)*(1 -$B21)</f>
         <v>80.224065750400001</v>
       </c>
-      <c r="AY23" s="9"/>
-      <c r="AZ23" s="6" t="s">
+      <c r="AY23" s="6"/>
+      <c r="AZ23" s="7" t="s">
         <v>405</v>
       </c>
-      <c r="BA23" s="6" t="s">
+      <c r="BA23" s="7" t="s">
         <v>415</v>
       </c>
-      <c r="BB23" s="6" t="s">
+      <c r="BB23" s="7" t="s">
         <v>416</v>
       </c>
-      <c r="BC23" s="6" t="s">
+      <c r="BC23" s="7" t="s">
         <v>406</v>
       </c>
     </row>
@@ -19070,16 +19072,16 @@
       <c r="AY26" s="5" t="s">
         <v>409</v>
       </c>
-      <c r="AZ26" s="8">
+      <c r="AZ26" s="11">
         <v>0.8</v>
       </c>
-      <c r="BA26" s="8">
+      <c r="BA26" s="11">
         <v>0.8</v>
       </c>
-      <c r="BB26" s="8">
+      <c r="BB26" s="11">
         <v>0.8</v>
       </c>
-      <c r="BC26" s="8">
+      <c r="BC26" s="11">
         <v>0.8</v>
       </c>
     </row>
@@ -19087,16 +19089,16 @@
       <c r="AY27" s="5" t="s">
         <v>410</v>
       </c>
-      <c r="AZ27" s="8">
+      <c r="AZ27" s="11">
         <v>0.19</v>
       </c>
-      <c r="BA27" s="8">
+      <c r="BA27" s="11">
         <v>0.23</v>
       </c>
-      <c r="BB27" s="8">
+      <c r="BB27" s="11">
         <v>0.19</v>
       </c>
-      <c r="BC27" s="8">
+      <c r="BC27" s="11">
         <v>0.23</v>
       </c>
     </row>
@@ -19104,16 +19106,16 @@
       <c r="AY28" s="5" t="s">
         <v>411</v>
       </c>
-      <c r="AZ28" s="8">
+      <c r="AZ28" s="11">
         <v>0.35</v>
       </c>
-      <c r="BA28" s="8">
+      <c r="BA28" s="11">
         <v>0.47</v>
       </c>
-      <c r="BB28" s="8">
+      <c r="BB28" s="11">
         <v>0.32</v>
       </c>
-      <c r="BC28" s="8">
+      <c r="BC28" s="11">
         <v>0.47</v>
       </c>
     </row>
@@ -19121,16 +19123,16 @@
       <c r="AY29" s="5" t="s">
         <v>412</v>
       </c>
-      <c r="AZ29" s="8">
+      <c r="AZ29" s="11">
         <v>0.18</v>
       </c>
-      <c r="BA29" s="8">
+      <c r="BA29" s="11">
         <v>0.15</v>
       </c>
-      <c r="BB29" s="8">
+      <c r="BB29" s="11">
         <v>0.18</v>
       </c>
-      <c r="BC29" s="8">
+      <c r="BC29" s="11">
         <v>0.15</v>
       </c>
     </row>

</xml_diff>